<commit_message>
docs(seo): add Discontinued-SOP SEO-treatment note to rev3 Summary
Documents SOP-PDP-DISC-001 v2.1 SEO handling for the 15 discontinued-SOP
candidates: keep URL self-canonical, no 301 by default, schema.org/Discontinued,
close hidden purchase paths, verify replacement SKU. No redirect proposed for
discontinued items.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MRQaWQFtdUDRDnv4iiLUx
</commit_message>
<xml_diff>
--- a/docs/seo/pages-blocked-crawling-report-2026-08-26-rev3.xlsx
+++ b/docs/seo/pages-blocked-crawling-report-2026-08-26-rev3.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -813,6 +813,13 @@
       </c>
       <c r="B28" s="12" t="n">
         <v>53</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>SEO treatment for the 15 Discontinued-SOP candidates (per SOP-PDP-DISC-001 v2.1): keep the historical URL live and self-canonical, NO 301 by default, apply the discontinued template + tag and schema.org/Discontinued availability, and close all hidden purchase paths; exact replacement SKU must be verified (or REPLACEMENT = PENDING). No redirect is proposed for discontinued items in this report.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>